<commit_message>
feat: implement dynamic area unit resolution, robust coordinate parsing, and improved area calculation logic
</commit_message>
<xml_diff>
--- a/sample_templates/Area_Audit_To_CA.xlsx
+++ b/sample_templates/Area_Audit_To_CA.xlsx
@@ -17,16 +17,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +34,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -45,21 +42,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,78 +413,59 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>CA_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>CA_Name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>area_Audit_DTO</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Latitude</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Longitude</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>audited_count</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>CA_Response</t>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Coordinates</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>sample_ca_uuid</t>
+          <t>sample_ca_1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Sample Area Name</t>
+          <t>Example - FeatureCollection</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>{"type": "FeatureCollection", "features": [{"type": "Feature", "geometry": {"type": "MultiPolygon", "coordinates": [[[[-113.59543, 33.78305], [-113.5935, 33.78305], [-113.59295, 33.78205], [-113.59295, 33.77967], [-113.59841, 33.78118], [-113.5985, 33.78305], [-113.59543, 33.78305]]]]}, "properties": {}}]}</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>sample_ca_2</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Example - Raw Coord Array</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
           <t>[[77.5, 12.9], [77.51, 12.9], [77.51, 12.91], [77.5, 12.9]]</t>
         </is>
       </c>
-      <c r="D2" t="n">
-        <v>12.9</v>
-      </c>
-      <c r="E2" t="n">
-        <v>77.5</v>
-      </c>
-      <c r="F2" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>